<commit_message>
DATA: Obtengo predicciones para los proximos 15 dias
</commit_message>
<xml_diff>
--- a/data/england/p4_modeling/2024-10-02/df_best_model.xlsx
+++ b/data/england/p4_modeling/2024-10-02/df_best_model.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W49"/>
+  <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,7 +496,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>% ROI 100</t>
+          <t>% roi_100</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -545,22 +545,22 @@
         <v>860</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.01440714299954607</v>
+        <v>-0.01440714299954692</v>
       </c>
       <c r="C2" t="n">
-        <v>1.127483283172962</v>
+        <v>1.127483283172959</v>
       </c>
       <c r="D2" t="n">
-        <v>1.186257825024301</v>
+        <v>1.186257825024297</v>
       </c>
       <c r="E2" t="n">
-        <v>34.93830479936172</v>
+        <v>34.93830479936162</v>
       </c>
       <c r="F2" t="n">
-        <v>8059.733334261385</v>
+        <v>15120.22078984523</v>
       </c>
       <c r="G2" t="n">
-        <v>40.0981757923452</v>
+        <v>71.32179617851524</v>
       </c>
       <c r="H2" t="n">
         <v>-0.5</v>
@@ -581,7 +581,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>(201, 31)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -590,31 +590,31 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>34.56431956977754</v>
+        <v>62.25751986122732</v>
       </c>
       <c r="P2" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q2" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="T2" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="U2" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="V2" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="W2" t="n">
-        <v>59.70149253731343</v>
+        <v>59.43396226415094</v>
       </c>
     </row>
     <row r="3">
@@ -622,22 +622,22 @@
         <v>432</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.7939613376487187</v>
+        <v>-0.7939613499550131</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03261274730908952</v>
+        <v>0.03261273677241519</v>
       </c>
       <c r="D3" t="n">
-        <v>2.363073037620655</v>
+        <v>2.363073006705503</v>
       </c>
       <c r="E3" t="n">
-        <v>5.288584788546756</v>
+        <v>5.28858472948063</v>
       </c>
       <c r="F3" t="n">
-        <v>1172.784544639944</v>
+        <v>1600.358117915456</v>
       </c>
       <c r="G3" t="n">
-        <v>5.834748978308181</v>
+        <v>7.548859046771017</v>
       </c>
       <c r="H3" t="n">
         <v>-0.5</v>
@@ -658,7 +658,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>(201, 16)</t>
+          <t>(212, 16)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -667,31 +667,31 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>177.9100722796811</v>
+        <v>230.4696586014843</v>
       </c>
       <c r="P3" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q3" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S3" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="T3" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="U3" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="V3" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="W3" t="n">
-        <v>58.70646766169154</v>
+        <v>58.01886792452831</v>
       </c>
     </row>
     <row r="4">
@@ -699,22 +699,22 @@
         <v>146</v>
       </c>
       <c r="B4" t="n">
-        <v>4.377337833343947</v>
+        <v>4.37733775852683</v>
       </c>
       <c r="C4" t="n">
-        <v>2.247064929702806</v>
+        <v>2.24706489160916</v>
       </c>
       <c r="D4" t="n">
-        <v>4.321306137648223</v>
+        <v>4.321306079130742</v>
       </c>
       <c r="E4" t="n">
-        <v>4.454701611156757</v>
+        <v>4.45470155302961</v>
       </c>
       <c r="F4" t="n">
-        <v>1017.36707213083</v>
+        <v>1128.249343001611</v>
       </c>
       <c r="G4" t="n">
-        <v>5.061527722043931</v>
+        <v>5.321930863215147</v>
       </c>
       <c r="H4" t="n">
         <v>-0.5</v>
@@ -735,7 +735,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>(201, 31)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -744,54 +744,54 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>1.252506216059081</v>
+        <v>1.368392155957733</v>
       </c>
       <c r="P4" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q4" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R4" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S4" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="T4" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="U4" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="V4" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="W4" t="n">
-        <v>59.20398009950249</v>
+        <v>58.49056603773585</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>682</v>
+        <v>1536</v>
       </c>
       <c r="B5" t="n">
-        <v>0.1635441624542409</v>
+        <v>0.1739890298160674</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.2439101372756677</v>
+        <v>-0.2301817734925082</v>
       </c>
       <c r="D5" t="n">
-        <v>1.129502923907369</v>
+        <v>0.4132464390111742</v>
       </c>
       <c r="E5" t="n">
-        <v>2.801562834467349</v>
+        <v>0.4808518048053221</v>
       </c>
       <c r="F5" t="n">
-        <v>637.530264528903</v>
+        <v>478.1157967186381</v>
       </c>
       <c r="G5" t="n">
-        <v>3.171792360840314</v>
+        <v>2.255263192069048</v>
       </c>
       <c r="H5" t="n">
         <v>-0.5</v>
@@ -812,7 +812,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>(201, 29)</t>
+          <t>(212, 25)</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -821,54 +821,54 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>14.00393823835025</v>
+        <v>10.79774878718819</v>
       </c>
       <c r="P5" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q5" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R5" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S5" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="T5" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="U5" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="V5" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="W5" t="n">
-        <v>59.20398009950249</v>
+        <v>57.54716981132076</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>288</v>
+        <v>682</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.2492399216360792</v>
+        <v>0.1635441466506455</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.4478210367301</v>
+        <v>-0.2439101427985219</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5291422953615397</v>
+        <v>1.129502910787259</v>
       </c>
       <c r="E6" t="n">
-        <v>1.772531250897064</v>
+        <v>2.8015628103511</v>
       </c>
       <c r="F6" t="n">
-        <v>399.7251791459742</v>
+        <v>449.3662063621945</v>
       </c>
       <c r="G6" t="n">
-        <v>1.988682483313304</v>
+        <v>2.119651916802804</v>
       </c>
       <c r="H6" t="n">
         <v>-0.5</v>
@@ -889,7 +889,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 29)</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -898,54 +898,54 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>5.440797372616229</v>
+        <v>9.690298371698749</v>
       </c>
       <c r="P6" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q6" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R6" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S6" t="n">
+        <v>85</v>
+      </c>
+      <c r="T6" t="n">
+        <v>54</v>
+      </c>
+      <c r="U6" t="n">
         <v>73</v>
       </c>
-      <c r="T6" t="n">
-        <v>62</v>
-      </c>
-      <c r="U6" t="n">
-        <v>66</v>
-      </c>
       <c r="V6" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="W6" t="n">
-        <v>58.2089552238806</v>
+        <v>58.01886792452831</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>1116</v>
+        <v>1130</v>
       </c>
       <c r="B7" t="n">
-        <v>-1.231315009587991</v>
+        <v>-0.5803498245424348</v>
       </c>
       <c r="C7" t="n">
-        <v>0.129382618057009</v>
+        <v>0.3604641000501758</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.2342559842448198</v>
+        <v>2.289475661871246</v>
       </c>
       <c r="E7" t="n">
-        <v>1.296064726840112</v>
+        <v>1.305861118498618</v>
       </c>
       <c r="F7" t="n">
-        <v>296.1484198068527</v>
+        <v>362.1455983199157</v>
       </c>
       <c r="G7" t="n">
-        <v>1.473375222919665</v>
+        <v>1.708233954339225</v>
       </c>
       <c r="H7" t="n">
         <v>-0.5</v>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -966,7 +966,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>(201, 27)</t>
+          <t>(212, 37)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -975,54 +975,54 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>10.38773696997275</v>
+        <v>3.738984975484223</v>
       </c>
       <c r="P7" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q7" t="n">
+        <v>55</v>
+      </c>
+      <c r="R7" t="n">
+        <v>63</v>
+      </c>
+      <c r="S7" t="n">
+        <v>94</v>
+      </c>
+      <c r="T7" t="n">
         <v>51</v>
       </c>
-      <c r="R7" t="n">
-        <v>62</v>
-      </c>
-      <c r="S7" t="n">
-        <v>83</v>
-      </c>
-      <c r="T7" t="n">
-        <v>44</v>
-      </c>
       <c r="U7" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="V7" t="n">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="W7" t="n">
-        <v>57.71144278606965</v>
+        <v>57.07547169811321</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>1130</v>
+        <v>811</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.5803497920887954</v>
+        <v>-0.2546242100158793</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3604641311508038</v>
+        <v>0.04290627187442211</v>
       </c>
       <c r="D8" t="n">
-        <v>2.28947572944957</v>
+        <v>-0.1015649524208972</v>
       </c>
       <c r="E8" t="n">
-        <v>1.305861159781158</v>
+        <v>1.048795160851438</v>
       </c>
       <c r="F8" t="n">
-        <v>293.68081251948</v>
+        <v>355.9142661576282</v>
       </c>
       <c r="G8" t="n">
-        <v>1.461098569748657</v>
+        <v>1.67884087810202</v>
       </c>
       <c r="H8" t="n">
         <v>-0.5</v>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>(201, 37)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1052,54 +1052,54 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>3.053381303387969</v>
+        <v>38.12809957051604</v>
       </c>
       <c r="P8" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q8" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R8" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S8" t="n">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="T8" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="U8" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="V8" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="W8" t="n">
-        <v>57.71144278606965</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>811</v>
+        <v>288</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.2546242100158798</v>
+        <v>-0.07583992964581711</v>
       </c>
       <c r="C9" t="n">
-        <v>0.04290627187442211</v>
+        <v>-0.288437096087221</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1015649524208973</v>
+        <v>0.6190369519895285</v>
       </c>
       <c r="E9" t="n">
-        <v>1.048795160851438</v>
+        <v>1.694591990741122</v>
       </c>
       <c r="F9" t="n">
-        <v>236.2262772706193</v>
+        <v>251.7959573595038</v>
       </c>
       <c r="G9" t="n">
-        <v>1.175255110799101</v>
+        <v>1.187716779997659</v>
       </c>
       <c r="H9" t="n">
         <v>-0.5</v>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>(201, 31)</t>
+          <t>(212, 25)</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1129,57 +1129,57 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>26.39121949907073</v>
+        <v>5.117767083740515</v>
       </c>
       <c r="P9" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q9" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R9" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S9" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="T9" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="U9" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="V9" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="W9" t="n">
-        <v>56.71641791044776</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>32</v>
+        <v>1116</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.4717589034227129</v>
+        <v>-1.011784388785441</v>
       </c>
       <c r="C10" t="n">
-        <v>0.2865445430127954</v>
+        <v>0.2471880434949603</v>
       </c>
       <c r="D10" t="n">
-        <v>1.99756985189969</v>
+        <v>-0.1058910324052047</v>
       </c>
       <c r="E10" t="n">
-        <v>1.016305209397624</v>
+        <v>1.311161708266124</v>
       </c>
       <c r="F10" t="n">
-        <v>229.3117038829864</v>
+        <v>220.0105477118452</v>
       </c>
       <c r="G10" t="n">
-        <v>1.140854248174062</v>
+        <v>1.037785602414364</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>(201, 10)</t>
+          <t>(212, 27)</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1206,57 +1206,57 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>2.981420257314473</v>
+        <v>3.198364887480986</v>
       </c>
       <c r="P10" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q10" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R10" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S10" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="T10" t="n">
         <v>48</v>
       </c>
       <c r="U10" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="V10" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="W10" t="n">
-        <v>55.72139303482587</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>14</v>
+        <v>235</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.7401069446195185</v>
+        <v>-0.7830270571640949</v>
       </c>
       <c r="C11" t="n">
-        <v>0.2864643308536782</v>
+        <v>-0.508661487376036</v>
       </c>
       <c r="D11" t="n">
-        <v>1.069073505157536</v>
+        <v>-0.2447138625329862</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8158824571187417</v>
+        <v>0.571322665474153</v>
       </c>
       <c r="F11" t="n">
-        <v>185.3277954205593</v>
+        <v>189.0125929521162</v>
       </c>
       <c r="G11" t="n">
-        <v>0.922028832938106</v>
+        <v>0.8915688346797935</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1264,7 +1264,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>(201, 8)</t>
+          <t>(212, 49)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1283,31 +1283,31 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>2.218651446727812</v>
+        <v>2.752774402636635</v>
       </c>
       <c r="P11" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q11" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S11" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="T11" t="n">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="U11" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="V11" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="W11" t="n">
-        <v>57.2139303482587</v>
+        <v>52.83018867924528</v>
       </c>
     </row>
     <row r="12">
@@ -1315,22 +1315,22 @@
         <v>872</v>
       </c>
       <c r="B12" t="n">
-        <v>1.306961621261062</v>
+        <v>1.306961642615121</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4270207402148176</v>
+        <v>0.4270207494295255</v>
       </c>
       <c r="D12" t="n">
-        <v>1.101279983980487</v>
+        <v>1.101279995396658</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7120179498822108</v>
+        <v>0.7120179577085802</v>
       </c>
       <c r="F12" t="n">
-        <v>161.6313307311958</v>
+        <v>158.5348573881058</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8041359737870436</v>
+        <v>0.7478059310759706</v>
       </c>
       <c r="H12" t="n">
         <v>-0.5</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>(201, 24)</t>
+          <t>(212, 24)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1360,57 +1360,57 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>0.883130953738954</v>
+        <v>0.7512168485372084</v>
       </c>
       <c r="P12" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q12" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R12" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S12" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T12" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="U12" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V12" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="W12" t="n">
-        <v>55.22388059701493</v>
+        <v>54.24528301886793</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>878</v>
+        <v>32</v>
       </c>
       <c r="B13" t="n">
-        <v>0.351498556397795</v>
+        <v>-0.2477645639389803</v>
       </c>
       <c r="C13" t="n">
-        <v>0.03390393877586916</v>
+        <v>0.3729790947000873</v>
       </c>
       <c r="D13" t="n">
-        <v>0.965017654738484</v>
+        <v>1.575801063664704</v>
       </c>
       <c r="E13" t="n">
-        <v>0.6269879987919765</v>
+        <v>0.9423361090441793</v>
       </c>
       <c r="F13" t="n">
-        <v>145.16351237746</v>
+        <v>153.3012430371957</v>
       </c>
       <c r="G13" t="n">
-        <v>0.7222065292410944</v>
+        <v>0.7231190709301683</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>(201, 8)</t>
+          <t>(212, 10)</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1437,57 +1437,57 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>20.30155242479139</v>
+        <v>0.938765687421781</v>
       </c>
       <c r="P13" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q13" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R13" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S13" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="T13" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="U13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="V13" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="W13" t="n">
-        <v>57.71144278606965</v>
+        <v>54.24528301886793</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>1390</v>
+        <v>878</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.6932879585861633</v>
+        <v>0.3514985338724523</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.6902056896992107</v>
+        <v>0.03390392887195474</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.5075357078022835</v>
+        <v>0.9650176391083446</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6641280346508924</v>
+        <v>0.6269879879963958</v>
       </c>
       <c r="F14" t="n">
-        <v>144.6019472600641</v>
+        <v>151.0900306019217</v>
       </c>
       <c r="G14" t="n">
-        <v>0.7194126729356422</v>
+        <v>0.7126888235939701</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 8)</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1514,54 +1514,54 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>2.042316346666397</v>
+        <v>20.02083290363156</v>
       </c>
       <c r="P14" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q14" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R14" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S14" t="n">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="T14" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="U14" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="V14" t="n">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="W14" t="n">
-        <v>55.22388059701493</v>
+        <v>57.07547169811321</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>320</v>
+        <v>504</v>
       </c>
       <c r="B15" t="n">
-        <v>-0.3763213469936971</v>
+        <v>2.259741504024007</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.679443511484252</v>
+        <v>0.4463224204891336</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.3067872217751226</v>
+        <v>0.537380097753947</v>
       </c>
       <c r="E15" t="n">
-        <v>0.5996212075370029</v>
+        <v>0.4244056962752481</v>
       </c>
       <c r="F15" t="n">
-        <v>132.8894618964754</v>
+        <v>150.8457782769085</v>
       </c>
       <c r="G15" t="n">
-        <v>0.6611416014750019</v>
+        <v>0.7115366899854173</v>
       </c>
       <c r="H15" t="n">
         <v>-0.5</v>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>(201, 20)</t>
+          <t>(212, 33)</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1591,57 +1591,57 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>1.973063382459464</v>
+        <v>0.5942212564755992</v>
       </c>
       <c r="P15" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q15" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R15" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S15" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="T15" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="U15" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="V15" t="n">
         <v>115</v>
       </c>
       <c r="W15" t="n">
-        <v>57.2139303482587</v>
+        <v>54.24528301886793</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>1536</v>
+        <v>1390</v>
       </c>
       <c r="B16" t="n">
-        <v>0.2526106788699121</v>
+        <v>-0.693287949860131</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.09342276888731874</v>
+        <v>-0.6902056876304493</v>
       </c>
       <c r="D16" t="n">
-        <v>0.486949360113767</v>
+        <v>-0.5075357067396301</v>
       </c>
       <c r="E16" t="n">
-        <v>0.583026150949884</v>
+        <v>0.6641280424247706</v>
       </c>
       <c r="F16" t="n">
-        <v>132.1648938800327</v>
+        <v>146.2821455776538</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6575367854727996</v>
+        <v>0.6900101206493104</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 25)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1668,57 +1668,57 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>8.03829262720615</v>
+        <v>1.999716654057415</v>
       </c>
       <c r="P16" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q16" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R16" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S16" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="T16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="U16" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="V16" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W16" t="n">
-        <v>56.71641791044776</v>
+        <v>54.71698113207547</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>235</v>
+        <v>798</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.7830270391426534</v>
+        <v>-0.8529832118195465</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.508661480100091</v>
+        <v>-0.589456623512797</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.2447138562845333</v>
+        <v>-0.1341239046070657</v>
       </c>
       <c r="E17" t="n">
-        <v>0.5713226813387452</v>
+        <v>0.5501731002880618</v>
       </c>
       <c r="F17" t="n">
-        <v>128.8770123131929</v>
+        <v>144.9272789186441</v>
       </c>
       <c r="G17" t="n">
-        <v>0.6411791657372784</v>
+        <v>0.6836192401822834</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>(201, 49)</t>
+          <t>(212, 11)</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1745,54 +1745,54 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>2.260522352923425</v>
+        <v>2.159744776652666</v>
       </c>
       <c r="P17" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q17" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R17" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S17" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="T17" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="U17" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="V17" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="W17" t="n">
-        <v>53.23383084577114</v>
+        <v>54.71698113207547</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>798</v>
+        <v>14</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.8529832118195461</v>
+        <v>-0.5103108969460655</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.589456623512797</v>
+        <v>0.3423567696060337</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.1341239046070657</v>
+        <v>0.9194961563669691</v>
       </c>
       <c r="E18" t="n">
-        <v>0.5501731002880611</v>
+        <v>0.7625137190571896</v>
       </c>
       <c r="F18" t="n">
-        <v>127.0667228940532</v>
+        <v>112.8889885593017</v>
       </c>
       <c r="G18" t="n">
-        <v>0.6321727507166823</v>
+        <v>0.53249522905331</v>
       </c>
       <c r="H18" t="n">
         <v>-0.5</v>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>(201, 11)</t>
+          <t>(212, 8)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1822,57 +1822,57 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>2.072466956006574</v>
+        <v>0.5553810420225597</v>
       </c>
       <c r="P18" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q18" t="n">
+        <v>55</v>
+      </c>
+      <c r="R18" t="n">
+        <v>63</v>
+      </c>
+      <c r="S18" t="n">
+        <v>87</v>
+      </c>
+      <c r="T18" t="n">
         <v>51</v>
       </c>
-      <c r="R18" t="n">
-        <v>62</v>
-      </c>
-      <c r="S18" t="n">
-        <v>79</v>
-      </c>
-      <c r="T18" t="n">
-        <v>55</v>
-      </c>
       <c r="U18" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="V18" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="W18" t="n">
-        <v>55.22388059701493</v>
+        <v>55.66037735849056</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>1006</v>
+        <v>222</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.777715839238856</v>
+        <v>-1.467001359729218</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.5849557700501804</v>
+        <v>-0.603924989932363</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1616793887510099</v>
+        <v>-0.3780185432578898</v>
       </c>
       <c r="E19" t="n">
-        <v>0.4657549560052323</v>
+        <v>0.1487620086959595</v>
       </c>
       <c r="F19" t="n">
-        <v>104.2700998634057</v>
+        <v>90.10291957026345</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5187567157383368</v>
+        <v>0.4250137715578465</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 20)</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1899,75 +1899,75 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>1.886830667032886</v>
+        <v>1.703752582924986</v>
       </c>
       <c r="P19" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q19" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R19" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S19" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="T19" t="n">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="U19" t="n">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="V19" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="W19" t="n">
-        <v>54.72636815920397</v>
+        <v>53.77358490566038</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>188</v>
+        <v>1444</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.3365863792498627</v>
+        <v>-0.0407761079964169</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.6202324521757625</v>
+        <v>-0.05351773379816763</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.06560119926392655</v>
+        <v>-0.3204116209545487</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4281752187083691</v>
+        <v>0.2337549432608508</v>
       </c>
       <c r="F20" t="n">
-        <v>96.73390892648442</v>
+        <v>80.09515712224521</v>
       </c>
       <c r="G20" t="n">
-        <v>0.4812632284899722</v>
+        <v>0.377807344916251</v>
       </c>
       <c r="H20" t="n">
         <v>-0.5</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>linear</t>
+          <t>kelly</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>(201, 31)</t>
+          <t>(212, 52)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1976,57 +1976,57 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>1.775940096010312</v>
+        <v>8.059479505262358</v>
       </c>
       <c r="P20" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q20" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R20" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S20" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="T20" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="U20" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="V20" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="W20" t="n">
-        <v>58.2089552238806</v>
+        <v>56.13207547169812</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>504</v>
+        <v>286</v>
       </c>
       <c r="B21" t="n">
-        <v>2.259741387705714</v>
+        <v>-0.6929083138764903</v>
       </c>
       <c r="C21" t="n">
-        <v>0.446322380995245</v>
+        <v>-0.3702779184334557</v>
       </c>
       <c r="D21" t="n">
-        <v>0.5373800648757397</v>
+        <v>-0.03914348168694384</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4244056710330369</v>
+        <v>0.1339735170831015</v>
       </c>
       <c r="F21" t="n">
-        <v>94.67175182199611</v>
+        <v>72.05476953115539</v>
       </c>
       <c r="G21" t="n">
-        <v>0.4710037404079409</v>
+        <v>0.3398809883545065</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>(201, 33)</t>
+          <t>(212, 25)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2053,57 +2053,57 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>0.05529939896282916</v>
+        <v>1.917907796912248</v>
       </c>
       <c r="P21" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q21" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R21" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S21" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="T21" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="U21" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="V21" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="W21" t="n">
-        <v>54.22885572139303</v>
+        <v>54.24528301886793</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B22" t="n">
-        <v>0.01530174795194085</v>
+        <v>-0.4969668445654574</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.1672041013104723</v>
+        <v>-0.02459951893825462</v>
       </c>
       <c r="D22" t="n">
-        <v>0.4213221520634361</v>
+        <v>0.4938559183090558</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3673192899749068</v>
+        <v>0.2457257743552296</v>
       </c>
       <c r="F22" t="n">
-        <v>83.58304311726155</v>
+        <v>71.58661150021589</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4158360354092615</v>
+        <v>0.3376726957557353</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>(201, 16)</t>
+          <t>(212, 16)</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2130,54 +2130,54 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>3.486996623588305</v>
+        <v>14.7268007802633</v>
       </c>
       <c r="P22" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q22" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R22" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S22" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="T22" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="U22" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="V22" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="W22" t="n">
-        <v>57.2139303482587</v>
+        <v>54.71698113207547</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>736</v>
+        <v>1022</v>
       </c>
       <c r="B23" t="n">
-        <v>0.7637935089223692</v>
+        <v>-0.1286581451772187</v>
       </c>
       <c r="C23" t="n">
-        <v>0.03577923962948035</v>
+        <v>0.04545178753173772</v>
       </c>
       <c r="D23" t="n">
-        <v>0.3791091387111946</v>
+        <v>-0.0111488191002914</v>
       </c>
       <c r="E23" t="n">
-        <v>0.3073661331233402</v>
+        <v>0.2714356614399307</v>
       </c>
       <c r="F23" t="n">
-        <v>73.19367522309142</v>
+        <v>65.4915621209114</v>
       </c>
       <c r="G23" t="n">
-        <v>0.3641476379258279</v>
+        <v>0.3089224628344877</v>
       </c>
       <c r="H23" t="n">
         <v>-0.5</v>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>(201, 14)</t>
+          <t>(212, 11)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2207,75 +2207,75 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>9.177623719699957</v>
+        <v>5.796706567784066</v>
       </c>
       <c r="P23" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q23" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R23" t="n">
+        <v>63</v>
+      </c>
+      <c r="S23" t="n">
+        <v>82</v>
+      </c>
+      <c r="T23" t="n">
+        <v>68</v>
+      </c>
+      <c r="U23" t="n">
         <v>62</v>
       </c>
-      <c r="S23" t="n">
-        <v>89</v>
-      </c>
-      <c r="T23" t="n">
-        <v>37</v>
-      </c>
-      <c r="U23" t="n">
-        <v>75</v>
-      </c>
       <c r="V23" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="W23" t="n">
-        <v>57.2139303482587</v>
+        <v>52.83018867924528</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>1068</v>
+        <v>1108</v>
       </c>
       <c r="B24" t="n">
-        <v>0.4302018060140065</v>
+        <v>-0.4037581981261786</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.3970899856683843</v>
+        <v>-0.2452972604927378</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.01456378783964482</v>
+        <v>-0.2023662931720209</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3120030024448919</v>
+        <v>0.2831630778167512</v>
       </c>
       <c r="F24" t="n">
-        <v>72.52740794218462</v>
+        <v>57.70797122427541</v>
       </c>
       <c r="G24" t="n">
-        <v>0.3608328753342518</v>
+        <v>0.2722074114352614</v>
       </c>
       <c r="H24" t="n">
         <v>-0.5</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>linear</t>
+          <t>kelly</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>(201, 29)</t>
+          <t>(212, 54)</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2284,57 +2284,57 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>1.908692962193181</v>
+        <v>2.109704245732171</v>
       </c>
       <c r="P24" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q24" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R24" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S24" t="n">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="T24" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="U24" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="V24" t="n">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="W24" t="n">
-        <v>54.72636815920397</v>
+        <v>56.13207547169812</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>1108</v>
+        <v>538</v>
       </c>
       <c r="B25" t="n">
-        <v>-0.5594326583660566</v>
+        <v>-1.005647437048534</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.4247710897924153</v>
+        <v>-0.6045647710451106</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.2517968937846158</v>
+        <v>-0.2899798717588846</v>
       </c>
       <c r="E25" t="n">
-        <v>0.2764035824744018</v>
+        <v>0.05071179522831869</v>
       </c>
       <c r="F25" t="n">
-        <v>69.38834780693077</v>
+        <v>57.09159188736257</v>
       </c>
       <c r="G25" t="n">
-        <v>0.3452156607309989</v>
+        <v>0.2692999617328423</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>(201, 54)</t>
+          <t>(212, 17)</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2361,57 +2361,57 @@
         </is>
       </c>
       <c r="O25" t="n">
-        <v>1.81270987839522</v>
+        <v>1.445444350432963</v>
       </c>
       <c r="P25" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q25" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R25" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S25" t="n">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="T25" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="U25" t="n">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="V25" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W25" t="n">
-        <v>57.2139303482587</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>1124</v>
+        <v>428</v>
       </c>
       <c r="B26" t="n">
-        <v>0.4654098593432531</v>
+        <v>0.4151018901164354</v>
       </c>
       <c r="C26" t="n">
-        <v>0.09365771248463674</v>
+        <v>0.2355751708638039</v>
       </c>
       <c r="D26" t="n">
-        <v>1.095845993100747</v>
+        <v>0.3421538872889486</v>
       </c>
       <c r="E26" t="n">
-        <v>0.2633599597315566</v>
+        <v>0.1244453345472203</v>
       </c>
       <c r="F26" t="n">
-        <v>60.37311219919707</v>
+        <v>53.79395350558867</v>
       </c>
       <c r="G26" t="n">
-        <v>0.3003637422845625</v>
+        <v>0.2537450637056069</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>(201, 74)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2438,57 +2438,57 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>2.207036925376893</v>
+        <v>0.07712991473243079</v>
       </c>
       <c r="P26" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q26" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R26" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S26" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="T26" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="U26" t="n">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="V26" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="W26" t="n">
-        <v>54.72636815920397</v>
+        <v>53.30188679245283</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>1022</v>
+        <v>736</v>
       </c>
       <c r="B27" t="n">
-        <v>-0.1286581530488442</v>
+        <v>0.7637934788388798</v>
       </c>
       <c r="C27" t="n">
-        <v>0.04545178313414212</v>
+        <v>0.03577922835517512</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.01114882185766637</v>
+        <v>0.3791091273280787</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2714356581949587</v>
+        <v>0.3073661243352784</v>
       </c>
       <c r="F27" t="n">
-        <v>59.32197324411749</v>
+        <v>52.8528473688319</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2951341952443656</v>
+        <v>0.2493058838152448</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>(201, 11)</t>
+          <t>(212, 14)</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2515,54 +2515,54 @@
         </is>
       </c>
       <c r="O27" t="n">
-        <v>5.493346902878031</v>
+        <v>5.967894369895909</v>
       </c>
       <c r="P27" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q27" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R27" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S27" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="T27" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="U27" t="n">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="V27" t="n">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="W27" t="n">
-        <v>53.73134328358209</v>
+        <v>56.13207547169812</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>312</v>
+        <v>1244</v>
       </c>
       <c r="B28" t="n">
-        <v>2.060186060805565</v>
+        <v>0.3676670426782513</v>
       </c>
       <c r="C28" t="n">
-        <v>0.2670191399406437</v>
+        <v>-0.1556602695183821</v>
       </c>
       <c r="D28" t="n">
-        <v>0.02479897683101484</v>
+        <v>-0.1496348515575622</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2564448318717531</v>
+        <v>0.218395101444997</v>
       </c>
       <c r="F28" t="n">
-        <v>59.13725333846958</v>
+        <v>52.82568822723422</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2942151907386546</v>
+        <v>0.2491777746567652</v>
       </c>
       <c r="H28" t="n">
         <v>-0.5</v>
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>(201, 58)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2592,31 +2592,31 @@
         </is>
       </c>
       <c r="O28" t="n">
-        <v>0.1018505669820387</v>
+        <v>2.600779540133968</v>
       </c>
       <c r="P28" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q28" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R28" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S28" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="T28" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="U28" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="V28" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W28" t="n">
-        <v>54.22885572139303</v>
+        <v>53.30188679245283</v>
       </c>
     </row>
     <row r="29">
@@ -2624,22 +2624,22 @@
         <v>430</v>
       </c>
       <c r="B29" t="n">
-        <v>0.1310420612229237</v>
+        <v>0.16876028776238</v>
       </c>
       <c r="C29" t="n">
-        <v>0.07330730366832924</v>
+        <v>0.1278669303496679</v>
       </c>
       <c r="D29" t="n">
-        <v>0.3444237023182937</v>
+        <v>0.3048622582769839</v>
       </c>
       <c r="E29" t="n">
-        <v>0.2490351085016073</v>
+        <v>0.2462325700145787</v>
       </c>
       <c r="F29" t="n">
-        <v>57.89022538721775</v>
+        <v>51.86361971609858</v>
       </c>
       <c r="G29" t="n">
-        <v>0.2880110715781978</v>
+        <v>0.2446397156419745</v>
       </c>
       <c r="H29" t="n">
         <v>-0.25</v>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>(201, 16)</t>
+          <t>(212, 16)</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2669,54 +2669,54 @@
         </is>
       </c>
       <c r="O29" t="n">
-        <v>2.928818237283312</v>
+        <v>0.9132367921320784</v>
       </c>
       <c r="P29" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q29" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R29" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S29" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="T29" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="U29" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="V29" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W29" t="n">
-        <v>54.22885572139303</v>
+        <v>53.30188679245283</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>144</v>
+        <v>1344</v>
       </c>
       <c r="B30" t="n">
-        <v>-0.4969668445654577</v>
+        <v>-1.074053701876283</v>
       </c>
       <c r="C30" t="n">
-        <v>-0.02459951893825504</v>
+        <v>-0.7119515664705193</v>
       </c>
       <c r="D30" t="n">
-        <v>0.4938559183090552</v>
+        <v>-0.171706863680007</v>
       </c>
       <c r="E30" t="n">
-        <v>0.2457257743552293</v>
+        <v>0.1499693835933621</v>
       </c>
       <c r="F30" t="n">
-        <v>54.25844700630677</v>
+        <v>50.07960099856484</v>
       </c>
       <c r="G30" t="n">
-        <v>0.2699425224194367</v>
+        <v>0.2362245330120983</v>
       </c>
       <c r="H30" t="n">
         <v>-0.5</v>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>(201, 16)</t>
+          <t>(212, 16)</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2746,61 +2746,61 @@
         </is>
       </c>
       <c r="O30" t="n">
-        <v>11.97348785953881</v>
+        <v>1.331798599985074</v>
       </c>
       <c r="P30" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q30" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R30" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S30" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="T30" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="U30" t="n">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="V30" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="W30" t="n">
-        <v>54.72636815920397</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>1444</v>
+        <v>1068</v>
       </c>
       <c r="B31" t="n">
-        <v>-0.04077611365652786</v>
+        <v>0.3627958699018708</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.05351773653251271</v>
+        <v>-0.2398394868794276</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.3204116219548642</v>
+        <v>0.0540864392726822</v>
       </c>
       <c r="E31" t="n">
-        <v>0.2337549411410649</v>
+        <v>0.2954452711959914</v>
       </c>
       <c r="F31" t="n">
-        <v>51.51492354580535</v>
+        <v>49.24778898741519</v>
       </c>
       <c r="G31" t="n">
-        <v>0.2562931519691808</v>
+        <v>0.2323008914500717</v>
       </c>
       <c r="H31" t="n">
         <v>-0.5</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>kelly</t>
+          <t>linear</t>
         </is>
       </c>
       <c r="J31" t="n">
@@ -2810,11 +2810,11 @@
         <v>0</v>
       </c>
       <c r="L31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>(201, 52)</t>
+          <t>(212, 29)</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2823,57 +2823,57 @@
         </is>
       </c>
       <c r="O31" t="n">
-        <v>5.788938557098344</v>
+        <v>1.968568163952311</v>
       </c>
       <c r="P31" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q31" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R31" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S31" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="T31" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="U31" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="V31" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W31" t="n">
-        <v>56.21890547263681</v>
+        <v>53.77358490566038</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>1244</v>
+        <v>96</v>
       </c>
       <c r="B32" t="n">
-        <v>0.3676670445018166</v>
+        <v>-0.6157982996324591</v>
       </c>
       <c r="C32" t="n">
-        <v>-0.1556602688680752</v>
+        <v>-0.423335985816666</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.1496348511593464</v>
+        <v>-0.03209723291310837</v>
       </c>
       <c r="E32" t="n">
-        <v>0.218395101998302</v>
+        <v>0.09117690555279716</v>
       </c>
       <c r="F32" t="n">
-        <v>48.72589225467803</v>
+        <v>45.57812128486276</v>
       </c>
       <c r="G32" t="n">
-        <v>0.2424173744013832</v>
+        <v>0.2149911381361451</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>(201, 31)</t>
+          <t>(212, 16)</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2900,54 +2900,54 @@
         </is>
       </c>
       <c r="O32" t="n">
-        <v>2.557349066426425</v>
+        <v>1.507849900171849</v>
       </c>
       <c r="P32" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q32" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R32" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S32" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="T32" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="U32" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="V32" t="n">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="W32" t="n">
-        <v>53.73134328358209</v>
+        <v>54.71698113207547</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>222</v>
+        <v>1124</v>
       </c>
       <c r="B33" t="n">
-        <v>-1.142575615678543</v>
+        <v>0.465409875565633</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.4168670395741868</v>
+        <v>0.09365771968089774</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.2422477508378706</v>
+        <v>1.095846004698069</v>
       </c>
       <c r="E33" t="n">
-        <v>0.2046289316789526</v>
+        <v>0.2633599647544605</v>
       </c>
       <c r="F33" t="n">
-        <v>47.76209612039793</v>
+        <v>45.50416745367187</v>
       </c>
       <c r="G33" t="n">
-        <v>0.2376223687581986</v>
+        <v>0.214642299309773</v>
       </c>
       <c r="H33" t="n">
         <v>-0.5</v>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>(201, 20)</t>
+          <t>(212, 74)</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2977,57 +2977,57 @@
         </is>
       </c>
       <c r="O33" t="n">
-        <v>1.570019565473251</v>
+        <v>1.291773705798979</v>
       </c>
       <c r="P33" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q33" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R33" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S33" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="T33" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="U33" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="V33" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="W33" t="n">
-        <v>54.22885572139303</v>
+        <v>54.24528301886793</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>848</v>
+        <v>224</v>
       </c>
       <c r="B34" t="n">
-        <v>0.1963920488699031</v>
+        <v>-0.02746183203828508</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.04265726318939485</v>
+        <v>-0.2923432632892404</v>
       </c>
       <c r="D34" t="n">
-        <v>-0.03201033208541437</v>
+        <v>0.06365993493743266</v>
       </c>
       <c r="E34" t="n">
-        <v>0.2046679151931022</v>
+        <v>0.1631782042849112</v>
       </c>
       <c r="F34" t="n">
-        <v>46.33388332557078</v>
+        <v>44.62716256285353</v>
       </c>
       <c r="G34" t="n">
-        <v>0.2305168324655263</v>
+        <v>0.210505483787045</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>(201, 10)</t>
+          <t>(212, 20)</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -3054,31 +3054,31 @@
         </is>
       </c>
       <c r="O34" t="n">
-        <v>6.403929254487094</v>
+        <v>1.720062714695682</v>
       </c>
       <c r="P34" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q34" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R34" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S34" t="n">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="T34" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="U34" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="V34" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W34" t="n">
-        <v>54.22885572139303</v>
+        <v>53.30188679245283</v>
       </c>
     </row>
     <row r="35">
@@ -3086,22 +3086,22 @@
         <v>830</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.9497284979862302</v>
+        <v>-0.9497284979862306</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.3639086960868848</v>
+        <v>-0.3639086960868855</v>
       </c>
       <c r="D35" t="n">
-        <v>0.03173275385625658</v>
+        <v>0.03173275385625601</v>
       </c>
       <c r="E35" t="n">
-        <v>0.1989841960055267</v>
+        <v>0.1989841960055264</v>
       </c>
       <c r="F35" t="n">
-        <v>45.06736366985777</v>
+        <v>44.54356487032405</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2242157396510337</v>
+        <v>0.2101111550486983</v>
       </c>
       <c r="H35" t="n">
         <v>-0.25</v>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>(201, 7)</t>
+          <t>(212, 7)</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3131,57 +3131,57 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>1.616131854121731</v>
+        <v>1.577373273318352</v>
       </c>
       <c r="P35" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q35" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R35" t="n">
+        <v>63</v>
+      </c>
+      <c r="S35" t="n">
+        <v>76</v>
+      </c>
+      <c r="T35" t="n">
+        <v>74</v>
+      </c>
+      <c r="U35" t="n">
         <v>62</v>
       </c>
-      <c r="S35" t="n">
-        <v>74</v>
-      </c>
-      <c r="T35" t="n">
-        <v>67</v>
-      </c>
-      <c r="U35" t="n">
-        <v>60</v>
-      </c>
       <c r="V35" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="W35" t="n">
-        <v>53.23383084577114</v>
+        <v>52.35849056603774</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>624</v>
+        <v>1486</v>
       </c>
       <c r="B36" t="n">
-        <v>0.5449561217506408</v>
+        <v>0.5447858610943705</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.1652030391529423</v>
+        <v>0.07199535553553332</v>
       </c>
       <c r="D36" t="n">
-        <v>0.01744686769885514</v>
+        <v>0.08307713609773619</v>
       </c>
       <c r="E36" t="n">
-        <v>0.1872951022256648</v>
+        <v>0.1619361600642397</v>
       </c>
       <c r="F36" t="n">
-        <v>42.26098284802032</v>
+        <v>44.23409005091298</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2102536460100513</v>
+        <v>0.2086513681646839</v>
       </c>
       <c r="H36" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 25)</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3208,57 +3208,57 @@
         </is>
       </c>
       <c r="O36" t="n">
-        <v>2.272698414557627</v>
+        <v>1.898122616558286</v>
       </c>
       <c r="P36" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q36" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R36" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S36" t="n">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="T36" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="U36" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="V36" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="W36" t="n">
-        <v>56.71641791044776</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>940</v>
+        <v>188</v>
       </c>
       <c r="B37" t="n">
-        <v>-0.4012889919723028</v>
+        <v>-0.1854789672994232</v>
       </c>
       <c r="C37" t="n">
-        <v>-0.1372232704430253</v>
+        <v>-0.4482276748766224</v>
       </c>
       <c r="D37" t="n">
-        <v>0.09326952053018098</v>
+        <v>0.004698062753131751</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1852696918538955</v>
+        <v>0.3465133665638223</v>
       </c>
       <c r="F37" t="n">
-        <v>42.08824092581887</v>
+        <v>42.88651180449995</v>
       </c>
       <c r="G37" t="n">
-        <v>0.2093942334617854</v>
+        <v>0.2022948670023582</v>
       </c>
       <c r="H37" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>(201, 22)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3285,57 +3285,57 @@
         </is>
       </c>
       <c r="O37" t="n">
-        <v>2.525938223056164</v>
+        <v>1.451321679452393</v>
       </c>
       <c r="P37" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q37" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R37" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S37" t="n">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="T37" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="U37" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="V37" t="n">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="W37" t="n">
-        <v>52.7363184079602</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>1344</v>
+        <v>940</v>
       </c>
       <c r="B38" t="n">
-        <v>-0.7707852449491687</v>
+        <v>-0.4012889969797729</v>
       </c>
       <c r="C38" t="n">
-        <v>-0.5394497008347374</v>
+        <v>-0.1372232731454079</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.07527671355180568</v>
+        <v>0.09326951814991521</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1695991431935332</v>
+        <v>0.1852696897074998</v>
       </c>
       <c r="F38" t="n">
-        <v>39.33934735769805</v>
+        <v>40.9368175449367</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1957181460581992</v>
+        <v>0.1930981959666826</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>(201, 16)</t>
+          <t>(212, 22)</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3362,31 +3362,31 @@
         </is>
       </c>
       <c r="O38" t="n">
-        <v>1.362810741678691</v>
+        <v>2.407182553954001</v>
       </c>
       <c r="P38" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q38" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R38" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S38" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="T38" t="n">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="U38" t="n">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="V38" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="W38" t="n">
-        <v>57.2139303482587</v>
+        <v>51.88679245283019</v>
       </c>
     </row>
     <row r="39">
@@ -3394,25 +3394,25 @@
         <v>16</v>
       </c>
       <c r="B39" t="n">
-        <v>-0.2122342418431137</v>
+        <v>-0.2122342465390761</v>
       </c>
       <c r="C39" t="n">
-        <v>0.07201969137001896</v>
+        <v>0.07201968855412247</v>
       </c>
       <c r="D39" t="n">
-        <v>0.4286902849463055</v>
+        <v>0.4286902820691088</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1582568708653348</v>
+        <v>0.1582568691362782</v>
       </c>
       <c r="F39" t="n">
-        <v>37.40216948939957</v>
+        <v>40.04896719568757</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1860804452208934</v>
+        <v>0.1889102226211678</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -3430,7 +3430,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>(201, 8)</t>
+          <t>(212, 8)</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3439,57 +3439,57 @@
         </is>
       </c>
       <c r="O39" t="n">
-        <v>1.583743996691948</v>
+        <v>1.623035817201606</v>
       </c>
       <c r="P39" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q39" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R39" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S39" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="T39" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="U39" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="V39" t="n">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="W39" t="n">
-        <v>53.23383084577114</v>
+        <v>52.83018867924528</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>302</v>
+        <v>1150</v>
       </c>
       <c r="B40" t="n">
-        <v>-0.69731860261689</v>
+        <v>-0.03034252368786554</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.6350549635865874</v>
+        <v>-0.01314188674484356</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.2656630332350596</v>
+        <v>0.07401303558742484</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1549713521000648</v>
+        <v>0.0547160816967866</v>
       </c>
       <c r="F40" t="n">
-        <v>37.00306088351252</v>
+        <v>39.24608833654253</v>
       </c>
       <c r="G40" t="n">
-        <v>0.1840948302662314</v>
+        <v>0.1851230581912383</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>(201, 16)</t>
+          <t>(212, 25)</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3516,54 +3516,54 @@
         </is>
       </c>
       <c r="O40" t="n">
-        <v>1.28988802674106</v>
+        <v>15.08649015057708</v>
       </c>
       <c r="P40" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q40" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R40" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S40" t="n">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="T40" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="U40" t="n">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="V40" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="W40" t="n">
-        <v>56.21890547263681</v>
+        <v>55.66037735849056</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>286</v>
+        <v>1422</v>
       </c>
       <c r="B41" t="n">
-        <v>-0.4435625427164129</v>
+        <v>-0.9083273785767918</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.2174389905937018</v>
+        <v>-0.3273017653187258</v>
       </c>
       <c r="D41" t="n">
-        <v>0.03322527768986381</v>
+        <v>0.1225452168408105</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1647695942969254</v>
+        <v>0.1099439227291289</v>
       </c>
       <c r="F41" t="n">
-        <v>36.42696111695574</v>
+        <v>38.37014067876942</v>
       </c>
       <c r="G41" t="n">
-        <v>0.1812286622734116</v>
+        <v>0.1809912296168369</v>
       </c>
       <c r="H41" t="n">
         <v>-0.25</v>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 19)</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3593,54 +3593,54 @@
         </is>
       </c>
       <c r="O41" t="n">
-        <v>1.83346901941818</v>
+        <v>1.552979692732754</v>
       </c>
       <c r="P41" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q41" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R41" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S41" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="T41" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="U41" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="V41" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="W41" t="n">
-        <v>54.22885572139303</v>
+        <v>52.35849056603774</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>224</v>
+        <v>158</v>
       </c>
       <c r="B42" t="n">
-        <v>-0.02746181906916945</v>
+        <v>-0.8047495383218353</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.2923432586365131</v>
+        <v>-0.3948169291997625</v>
       </c>
       <c r="D42" t="n">
-        <v>0.06365993973921083</v>
+        <v>0.00258055592359805</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1631782086451997</v>
+        <v>0.1141223515357377</v>
       </c>
       <c r="F42" t="n">
-        <v>36.27371731672054</v>
+        <v>37.7774304796755</v>
       </c>
       <c r="G42" t="n">
-        <v>0.1804662553070673</v>
+        <v>0.1781954267909222</v>
       </c>
       <c r="H42" t="n">
         <v>-0.5</v>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>(201, 20)</t>
+          <t>(212, 8)</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3670,54 +3670,54 @@
         </is>
       </c>
       <c r="O42" t="n">
-        <v>1.617309446945213</v>
+        <v>1.451336844020592</v>
       </c>
       <c r="P42" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q42" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R42" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S42" t="n">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="T42" t="n">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="U42" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="V42" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="W42" t="n">
-        <v>53.73134328358209</v>
+        <v>56.60377358490566</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>1316</v>
+        <v>848</v>
       </c>
       <c r="B43" t="n">
-        <v>0.7606730248468597</v>
+        <v>0.1963920412596173</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.1003915968367077</v>
+        <v>-0.04265726650649498</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1143587603080978</v>
+        <v>-0.03201033428443718</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1270600714607411</v>
+        <v>0.2046679127514962</v>
       </c>
       <c r="F43" t="n">
-        <v>30.83770033424639</v>
+        <v>37.56765304240804</v>
       </c>
       <c r="G43" t="n">
-        <v>0.1534213946977432</v>
+        <v>0.1772059105773964</v>
       </c>
       <c r="H43" t="n">
         <v>-0.25</v>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>(201, 43)</t>
+          <t>(212, 10)</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3747,54 +3747,54 @@
         </is>
       </c>
       <c r="O43" t="n">
-        <v>2.528229448798303</v>
+        <v>5.154178762261176</v>
       </c>
       <c r="P43" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q43" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R43" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S43" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="T43" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="U43" t="n">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="V43" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="W43" t="n">
-        <v>54.72636815920397</v>
+        <v>53.30188679245283</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>1456</v>
+        <v>154</v>
       </c>
       <c r="B44" t="n">
-        <v>-0.4724414407366854</v>
+        <v>0.07322845339175529</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.3818895335382935</v>
+        <v>-0.06175034448523149</v>
       </c>
       <c r="D44" t="n">
-        <v>0.05465301318190948</v>
+        <v>0.3350180514159409</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1237939878299079</v>
+        <v>0.3079554282547646</v>
       </c>
       <c r="F44" t="n">
-        <v>29.90546061436581</v>
+        <v>34.39829348971884</v>
       </c>
       <c r="G44" t="n">
-        <v>0.1487833861411234</v>
+        <v>0.1622561013665983</v>
       </c>
       <c r="H44" t="n">
         <v>-0.25</v>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>(201, 13)</t>
+          <t>(212, 16)</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3824,57 +3824,57 @@
         </is>
       </c>
       <c r="O44" t="n">
-        <v>1.389597967670419</v>
+        <v>3.62761451323408</v>
       </c>
       <c r="P44" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q44" t="n">
+        <v>55</v>
+      </c>
+      <c r="R44" t="n">
+        <v>63</v>
+      </c>
+      <c r="S44" t="n">
+        <v>94</v>
+      </c>
+      <c r="T44" t="n">
         <v>51</v>
       </c>
-      <c r="R44" t="n">
-        <v>62</v>
-      </c>
-      <c r="S44" t="n">
-        <v>85</v>
-      </c>
-      <c r="T44" t="n">
-        <v>41</v>
-      </c>
       <c r="U44" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="V44" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="W44" t="n">
-        <v>57.2139303482587</v>
+        <v>55.66037735849056</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>1038</v>
+        <v>148</v>
       </c>
       <c r="B45" t="n">
-        <v>-0.2879815865865049</v>
+        <v>-0.2106776835639741</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.1458736041970225</v>
+        <v>-0.05776385515527295</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.01059916995141142</v>
+        <v>0.2908013751570968</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1029920310823041</v>
+        <v>0.2259571090915757</v>
       </c>
       <c r="F45" t="n">
-        <v>26.99374294374715</v>
+        <v>34.39629875696286</v>
       </c>
       <c r="G45" t="n">
-        <v>0.1342972285758565</v>
+        <v>0.1622466922498248</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -3892,7 +3892,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>(201, 19)</t>
+          <t>(212, 31)</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3901,57 +3901,57 @@
         </is>
       </c>
       <c r="O45" t="n">
-        <v>1.920641053020597</v>
+        <v>3.808792657860097</v>
       </c>
       <c r="P45" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q45" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R45" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S45" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="T45" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="U45" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="V45" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="W45" t="n">
-        <v>56.71641791044776</v>
+        <v>56.13207547169812</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>60</v>
+        <v>272</v>
       </c>
       <c r="B46" t="n">
-        <v>0.7568123179926477</v>
+        <v>-0.1517574622436499</v>
       </c>
       <c r="C46" t="n">
-        <v>0.02193867746724479</v>
+        <v>-0.1488331743527213</v>
       </c>
       <c r="D46" t="n">
-        <v>0.178042021396518</v>
+        <v>-0.03245133136793962</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1051047715918767</v>
+        <v>0.05128624266139908</v>
       </c>
       <c r="F46" t="n">
-        <v>26.11427423963519</v>
+        <v>32.89659059397869</v>
       </c>
       <c r="G46" t="n">
-        <v>0.1299217623862448</v>
+        <v>0.1551725971414089</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>(201, 14)</t>
+          <t>(212, 19)</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3978,54 +3978,54 @@
         </is>
       </c>
       <c r="O46" t="n">
-        <v>4.922041680963792</v>
+        <v>2.042594151581177</v>
       </c>
       <c r="P46" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q46" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R46" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S46" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="T46" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="U46" t="n">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="V46" t="n">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="W46" t="n">
-        <v>52.7363184079602</v>
+        <v>54.24528301886793</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>1152</v>
+        <v>552</v>
       </c>
       <c r="B47" t="n">
-        <v>-0.1323619893837537</v>
+        <v>-0.4129970092220722</v>
       </c>
       <c r="C47" t="n">
-        <v>-0.1821812080403123</v>
+        <v>-0.144654834260073</v>
       </c>
       <c r="D47" t="n">
-        <v>0.2915643157148817</v>
+        <v>-0.115758168897428</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1011687329085016</v>
+        <v>0.05732069603875665</v>
       </c>
       <c r="F47" t="n">
-        <v>25.32149819652165</v>
+        <v>32.63271816680404</v>
       </c>
       <c r="G47" t="n">
-        <v>0.1259776029677694</v>
+        <v>0.1539279158811511</v>
       </c>
       <c r="H47" t="n">
         <v>-0.25</v>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>(201, 25)</t>
+          <t>(212, 32)</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -4055,57 +4055,57 @@
         </is>
       </c>
       <c r="O47" t="n">
-        <v>1.691496144541393</v>
+        <v>2.064104885733761</v>
       </c>
       <c r="P47" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q47" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R47" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S47" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="T47" t="n">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="U47" t="n">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="V47" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="W47" t="n">
-        <v>56.71641791044776</v>
+        <v>52.83018867924528</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>1262</v>
+        <v>352</v>
       </c>
       <c r="B48" t="n">
-        <v>0.3231349968814814</v>
+        <v>-0.4985802892517043</v>
       </c>
       <c r="C48" t="n">
-        <v>-0.04073676429231483</v>
+        <v>-0.4293087545344865</v>
       </c>
       <c r="D48" t="n">
-        <v>0.09707344678512414</v>
+        <v>-0.04201312539670841</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1048974161138559</v>
+        <v>0.06743936027075378</v>
       </c>
       <c r="F48" t="n">
-        <v>25.05039310369686</v>
+        <v>32.33363746501348</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1246288214114272</v>
+        <v>0.1525171578538372</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>(201, 9)</t>
+          <t>(212, 15)</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -4132,54 +4132,54 @@
         </is>
       </c>
       <c r="O48" t="n">
-        <v>4.059369676912189</v>
+        <v>1.355262165616018</v>
       </c>
       <c r="P48" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q48" t="n">
+        <v>55</v>
+      </c>
+      <c r="R48" t="n">
+        <v>63</v>
+      </c>
+      <c r="S48" t="n">
+        <v>93</v>
+      </c>
+      <c r="T48" t="n">
         <v>51</v>
       </c>
-      <c r="R48" t="n">
-        <v>62</v>
-      </c>
-      <c r="S48" t="n">
-        <v>85</v>
-      </c>
-      <c r="T48" t="n">
-        <v>38</v>
-      </c>
       <c r="U48" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="V48" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="W48" t="n">
-        <v>54.72636815920397</v>
+        <v>55.18867924528303</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>538</v>
+        <v>60</v>
       </c>
       <c r="B49" t="n">
-        <v>-0.713684380233351</v>
+        <v>0.7568123562228755</v>
       </c>
       <c r="C49" t="n">
-        <v>-0.4305496961202628</v>
+        <v>0.02193869163902832</v>
       </c>
       <c r="D49" t="n">
-        <v>-0.1742021451962037</v>
+        <v>0.1780420331105563</v>
       </c>
       <c r="E49" t="n">
-        <v>0.09861989274956358</v>
+        <v>0.1051047799831964</v>
       </c>
       <c r="F49" t="n">
-        <v>24.44908472161646</v>
+        <v>27.19730425012992</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1216372374209774</v>
+        <v>0.1282891709911789</v>
       </c>
       <c r="H49" t="n">
         <v>-0.25</v>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>(201, 17)</t>
+          <t>(212, 14)</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -4209,31 +4209,185 @@
         </is>
       </c>
       <c r="O49" t="n">
-        <v>1.282516138130083</v>
+        <v>4.847621777178182</v>
       </c>
       <c r="P49" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q49" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R49" t="n">
+        <v>63</v>
+      </c>
+      <c r="S49" t="n">
+        <v>78</v>
+      </c>
+      <c r="T49" t="n">
+        <v>72</v>
+      </c>
+      <c r="U49" t="n">
         <v>62</v>
       </c>
-      <c r="S49" t="n">
-        <v>84</v>
-      </c>
-      <c r="T49" t="n">
-        <v>35</v>
-      </c>
-      <c r="U49" t="n">
-        <v>82</v>
-      </c>
       <c r="V49" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="W49" t="n">
-        <v>56.71641791044776</v>
+        <v>52.35849056603774</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>440</v>
+      </c>
+      <c r="B50" t="n">
+        <v>-0.4521688640083241</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-0.2628700546787339</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-0.236740638886616</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.003378225223045348</v>
+      </c>
+      <c r="F50" t="n">
+        <v>25.86240264648263</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.1219924653135973</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>10</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="b">
+        <v>0</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>(212, 22)</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="O50" t="n">
+        <v>1.464078974163452</v>
+      </c>
+      <c r="P50" t="n">
+        <v>94</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>55</v>
+      </c>
+      <c r="R50" t="n">
+        <v>63</v>
+      </c>
+      <c r="S50" t="n">
+        <v>66</v>
+      </c>
+      <c r="T50" t="n">
+        <v>66</v>
+      </c>
+      <c r="U50" t="n">
+        <v>80</v>
+      </c>
+      <c r="V50" t="n">
+        <v>109</v>
+      </c>
+      <c r="W50" t="n">
+        <v>51.41509433962265</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>924</v>
+      </c>
+      <c r="B51" t="n">
+        <v>-0.07575158239418585</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.01602335571755773</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.3475549218291498</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.07472548341667093</v>
+      </c>
+      <c r="F51" t="n">
+        <v>23.65607387293355</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.1115852541176111</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>10</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="b">
+        <v>0</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>(212, 16)</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="O51" t="n">
+        <v>5.963912933377656</v>
+      </c>
+      <c r="P51" t="n">
+        <v>94</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>55</v>
+      </c>
+      <c r="R51" t="n">
+        <v>63</v>
+      </c>
+      <c r="S51" t="n">
+        <v>92</v>
+      </c>
+      <c r="T51" t="n">
+        <v>40</v>
+      </c>
+      <c r="U51" t="n">
+        <v>80</v>
+      </c>
+      <c r="V51" t="n">
+        <v>118</v>
+      </c>
+      <c r="W51" t="n">
+        <v>55.66037735849056</v>
       </c>
     </row>
   </sheetData>

</xml_diff>